<commit_message>
Aplicar logo oficial aos modelos de gestão e suas prévias
</commit_message>
<xml_diff>
--- a/public/modelos/PCMD-01-Controle-Documental-Exemplo.xlsx
+++ b/public/modelos/PCMD-01-Controle-Documental-Exemplo.xlsx
@@ -623,7 +623,7 @@
       <row>0</row>
       <rowOff>142875</rowOff>
     </from>
-    <ext cx="2381250" cy="552450"/>
+    <ext cx="1908746" cy="552450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -653,7 +653,7 @@
       <row>0</row>
       <rowOff>228600</rowOff>
     </from>
-    <ext cx="1628775" cy="371475"/>
+    <ext cx="1283467" cy="371475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -683,7 +683,7 @@
       <row>0</row>
       <rowOff>238125</rowOff>
     </from>
-    <ext cx="1581150" cy="361950"/>
+    <ext cx="1250558" cy="361950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -713,7 +713,7 @@
       <row>0</row>
       <rowOff>142875</rowOff>
     </from>
-    <ext cx="2362200" cy="542925"/>
+    <ext cx="1875836" cy="542925"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -743,7 +743,7 @@
       <row>0</row>
       <rowOff>161925</rowOff>
     </from>
-    <ext cx="2209800" cy="514350"/>
+    <ext cx="1777108" cy="514350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>

</xml_diff>